<commit_message>
Añadiendo ref a compañías importando y demás así como los evaluadores por compañía
</commit_message>
<xml_diff>
--- a/krm/static/files/import_companies_en.xlsx
+++ b/krm/static/files/import_companies_en.xlsx
@@ -5,12 +5,12 @@
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bienvenidosaez/Bitbucket/krm-kpmg/krm/static/files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bienvenidosaez/Bitbucket/krc-kpmg/krc/static/assets/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F17A1CFC-9804-7D4B-AB60-0855329C0F39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DED4B117-4E17-B346-BC68-DC774E1BF1D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="20480" windowHeight="23880" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="20480" windowHeight="24100" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Companies" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="507">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="508">
   <si>
     <t>VAT</t>
   </si>
@@ -1553,6 +1553,9 @@
     <t>ADDRESS</t>
   </si>
   <si>
+    <t>CICY</t>
+  </si>
+  <si>
     <t>POSTAL CODE</t>
   </si>
   <si>
@@ -1565,7 +1568,7 @@
     <t>CODE</t>
   </si>
   <si>
-    <t>CITY</t>
+    <t>REF</t>
   </si>
 </sst>
 </file>
@@ -2065,41 +2068,43 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="7.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="32.5" style="2" customWidth="1"/>
-    <col min="2" max="2" width="14.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.1640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="31" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="26.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.1640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="32.5" style="2" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="29.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.33203125" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="9" t="s">
-        <v>504</v>
-      </c>
-      <c r="B1" s="10"/>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1"/>
+      <c r="B1" s="9" t="s">
+        <v>505</v>
+      </c>
       <c r="C1" s="10"/>
       <c r="D1" s="10"/>
       <c r="E1" s="10"/>
       <c r="F1" s="10"/>
       <c r="G1" s="10"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H1" s="10"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>507</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>500</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>501</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>506</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>502</v>
@@ -2108,20 +2113,23 @@
         <v>503</v>
       </c>
       <c r="G2" s="1" t="s">
+        <v>504</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="D3" s="3"/>
-      <c r="G3" s="3"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="D4" s="3"/>
-      <c r="G4" s="3"/>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E3" s="3"/>
+      <c r="H3" s="3"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E4" s="3"/>
+      <c r="H4" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
@@ -2130,9 +2138,9 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{1D5701C4-C796-2344-99F1-75AE5206539D}">
           <x14:formula1>
-            <xm:f>'Country Codes'!A2:A250</xm:f>
+            <xm:f>'Country Codes'!B2:B250</xm:f>
           </x14:formula1>
-          <xm:sqref>F3:F820</xm:sqref>
+          <xm:sqref>G3:G820</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2151,10 +2159,10 @@
   <sheetData>
     <row r="1" spans="1:2" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="21" x14ac:dyDescent="0.25">
@@ -2557,7 +2565,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="22" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:2" ht="21" x14ac:dyDescent="0.25">
       <c r="A52" s="7" t="s">
         <v>103</v>
       </c>

</xml_diff>